<commit_message>
chore(tm): register the archival commits and ledger row 15
改动-0003/0004 covered; 账本 row 15 records the archive sealing; 27/26 clarify baseline commit 8a5c71d versus tag tm-v3.4 (38e02f7).
</commit_message>
<xml_diff>
--- a/协作/14-改动清单.xlsx
+++ b/协作/14-改动清单.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -599,6 +599,90 @@
         </is>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>已合并</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>改动-0003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>切片-0002</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>契约-0003</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>协作/**</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>归档层实例落库（26/28/29/30/31/32/33/34/36/37）、证据-0006</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>8a5c71d</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>已合并</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>改动-0004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>切片-0002</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>契约-0003</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>协作/26,27,归档/**</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>首次归档快照 快照-0001（dcg-tm-v3.4.zip，197 份文件，SHA256 f93cc611…）与证据-0007；标签 tm-v3.4</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>38e02f7</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>已合并</t>
         </is>

</xml_diff>

<commit_message>
chore(tm): register 改动-0005 and ledger row 16
</commit_message>
<xml_diff>
--- a/协作/14-改动清单.xlsx
+++ b/协作/14-改动清单.xlsx
@@ -83,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -100,6 +100,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -465,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -685,6 +686,48 @@
       <c r="H5" t="inlineStr">
         <is>
           <t>已合并</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>改动-0005</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>切片-0002</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>契约-0003</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>TEAMODEL.md</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>附录 B 版本历史按版本号排序（3.3 与 3.4 两行位置对调，内容不变）；便于交付给外部项目时阅读</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>3508ff6</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>已提交</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(tm): record the v3.5 rollout in the ledger and change list
</commit_message>
<xml_diff>
--- a/协作/14-改动清单.xlsx
+++ b/协作/14-改动清单.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -768,6 +768,48 @@
         </is>
       </c>
       <c r="H7" t="inlineStr">
+        <is>
+          <t>已提交</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>改动-0007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>切片-0003</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>契约-0005</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>协作/**（37+3 交付物与记录）;协作/归档/dcg-tm-v3.5.zip</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>按协议 v3.5 全开落地：补齐 14 份缺交付物、重写 01 画像为九角色全开、追加 15 类记录、生成证据-0008..0011、写入快照-0002</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>77fb43c</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>已提交</t>
         </is>

</xml_diff>

<commit_message>
chore(tm): record the protocol externalisation snapshot (snapshot-0003)
</commit_message>
<xml_diff>
--- a/协作/14-改动清单.xlsx
+++ b/协作/14-改动清单.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -810,6 +810,48 @@
         </is>
       </c>
       <c r="H8" t="inlineStr">
+        <is>
+          <t>已提交</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>改动-0008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>切片-0004</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>契约-0006</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>TEAMODEL.md;协作/模板/**;docs/TEAMODEL_draft_v1.md;协作/**</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>协议与模板移出 DCG，改由 https://github.com/CL98K/TEAMODEL.git (tag tm-v3.5.1) 维护；DCG 保留记录与本地模板缓存（.gitignore 排除）</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0436ca2</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>已提交</t>
         </is>

</xml_diff>